<commit_message>
feat(sellout): objetivo abierto por Grupo PBP (subgrupos con objetivo y alcance)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/OBJSELLOUT.xlsx
+++ b/01_INPUTS/OBJSELLOUT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2606D1C4-2930-4E72-91FF-776D699917C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B583E0-A355-4ADC-8504-47FB846FB997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B81FE791-F8CF-43A3-8CF6-56398690978F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
   <si>
     <t>categoria</t>
   </si>
@@ -64,13 +64,46 @@
   </si>
   <si>
     <t>SELL OUT</t>
+  </si>
+  <si>
+    <t>Grupo PBP</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>Medio Alto</t>
+  </si>
+  <si>
+    <t>Superior</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Nacionales</t>
+  </si>
+  <si>
+    <t>Importados</t>
+  </si>
+  <si>
+    <t>rtd (s)</t>
+  </si>
+  <si>
+    <t>RTD</t>
+  </si>
+  <si>
+    <t>ESPUMANTES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,16 +111,72 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -95,16 +184,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -421,87 +549,205 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EADD3D7B-52D7-447F-9122-8C994E3406C1}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4">
+        <v>10711</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4">
+        <v>338</v>
+      </c>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4111</v>
+      </c>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1863</v>
+      </c>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="4">
         <v>17023</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5">
         <v>817</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="6">
+        <v>678</v>
+      </c>
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="6">
+        <v>16341</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="6">
         <v>17019</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="7">
+        <v>4028</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="7">
+        <v>5028</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="7">
         <v>9056</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B15" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="8">
         <v>747</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="9">
         <v>425</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B17" s="10"/>
+      <c r="C17" s="10">
         <v>45087</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data(sell out): objetivos por categoría del mes actualizados en OBJSELLOUT.xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/OBJSELLOUT.xlsx
+++ b/01_INPUTS/OBJSELLOUT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B583E0-A355-4ADC-8504-47FB846FB997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008B498B-FC0C-4B5C-8D69-55D94617EF90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B81FE791-F8CF-43A3-8CF6-56398690978F}"/>
   </bookViews>
@@ -203,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -211,30 +211,31 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,189 +559,191 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4">
-        <v>10711</v>
+      <c r="C3" s="3">
+        <v>13335</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="4">
-        <v>338</v>
+      <c r="C4" s="3">
+        <v>368</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4">
-        <v>4111</v>
+      <c r="C5" s="3">
+        <v>4499</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="4">
-        <v>1863</v>
+      <c r="C6" s="3">
+        <v>2030</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="4">
-        <v>17023</v>
+      <c r="C7" s="3">
+        <v>20232</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="5">
-        <v>817</v>
+      <c r="C8" s="4">
+        <v>809</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="6">
-        <v>678</v>
+      <c r="C9" s="5">
+        <v>1399</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="6">
-        <v>16341</v>
+      <c r="C10" s="5">
+        <v>18115</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="6">
-        <v>17019</v>
+      <c r="C11" s="5">
+        <v>19514</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="7">
-        <v>4028</v>
-      </c>
+      <c r="C12" s="6">
+        <v>5525</v>
+      </c>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="7">
-        <v>5028</v>
-      </c>
+      <c r="C13" s="6">
+        <v>6752</v>
+      </c>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="7">
-        <v>9056</v>
+      <c r="C14" s="6">
+        <v>12277</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="8">
-        <v>747</v>
+      <c r="C15" s="7">
+        <v>996</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="9">
-        <v>425</v>
+      <c r="C16" s="8">
+        <v>457</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10">
-        <v>45087</v>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9">
+        <v>54283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-04_1711 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/OBJSELLOUT.xlsx
+++ b/01_INPUTS/OBJSELLOUT.xlsx
@@ -8,14 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87CA28C-ECB4-4F34-9699-E3BC7F03DF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72A0308-DBA3-46B6-8EA6-004008EC1AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -93,7 +104,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -219,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -249,30 +260,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -598,11 +612,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="13"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -622,8 +636,8 @@
       <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="15">
-        <v>13062.458845678639</v>
+      <c r="C3" s="11">
+        <v>13217.150326380846</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -633,8 +647,8 @@
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="14">
-        <v>368.58332722913599</v>
+      <c r="C4" s="18">
+        <v>365.15940424038524</v>
       </c>
       <c r="D4" s="1"/>
     </row>
@@ -645,8 +659,8 @@
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="14">
-        <v>4487.78289326905</v>
+      <c r="C5" s="18">
+        <v>4462.8536073903924</v>
       </c>
       <c r="D5" s="1"/>
     </row>
@@ -657,8 +671,8 @@
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="14">
-        <v>2165.4765764815538</v>
+      <c r="C6" s="18">
+        <v>2466.3693174301065</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -669,8 +683,9 @@
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3">
-        <v>20084.3</v>
+      <c r="C7" s="11">
+        <f>SUM(C3:C6)</f>
+        <v>20511.532655441733</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -681,8 +696,8 @@
       <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="16">
-        <v>338.56904349286151</v>
+      <c r="C8" s="20">
+        <v>1372.2704956991149</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -693,7 +708,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="17">
-        <v>764.95250462048648</v>
+        <v>489.01923646361087</v>
       </c>
       <c r="D9" s="1"/>
     </row>
@@ -705,7 +720,7 @@
         <v>13</v>
       </c>
       <c r="C10" s="17">
-        <v>24379.552985127426</v>
+        <v>26540.575745363996</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -715,8 +730,9 @@
       <c r="B11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="5">
-        <v>25144.51</v>
+      <c r="C11" s="17">
+        <f>SUM(C9:C10)</f>
+        <v>27029.594981827606</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -726,9 +742,7 @@
       <c r="B12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="18">
-        <v>13886.903939532236</v>
-      </c>
+      <c r="C12" s="19"/>
       <c r="D12" s="10"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -738,9 +752,7 @@
       <c r="B13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="6">
-        <v>6752</v>
-      </c>
+      <c r="C13" s="6"/>
       <c r="D13" s="10"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -750,8 +762,8 @@
       <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="6">
-        <v>12277</v>
+      <c r="C14" s="19">
+        <v>14543.321694671846</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -761,8 +773,8 @@
       <c r="B15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="19">
-        <v>1612.0353353065727</v>
+      <c r="C15" s="16">
+        <v>1478.3740365045551</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -772,8 +784,8 @@
       <c r="B16" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="8">
-        <v>527</v>
+      <c r="C16" s="15">
+        <v>656.55243169487835</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -783,8 +795,8 @@
       <c r="B17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="4">
-        <v>6050</v>
+      <c r="C17" s="20">
+        <v>6346.5261243215537</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,8 +804,8 @@
         <v>21</v>
       </c>
       <c r="B18" s="9"/>
-      <c r="C18" s="20">
-        <v>67643.372130179487</v>
+      <c r="C18" s="21">
+        <v>71938.172420161281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>